<commit_message>
📊 Horarios actualizados Línea 141
</commit_message>
<xml_diff>
--- a/horarios-141-2026-01-08.xlsx
+++ b/horarios-141-2026-01-08.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LP1912" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="LP1912-215" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="6203-6173" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LP1912" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LP1912-215" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6203-6173" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,14 +441,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:01:27</t>
+          <t>Última actualización: 19:42:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Ejecuciones: 15 filas únicas</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -849,6 +849,481 @@
         <v>90</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>8</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>19:51</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>9</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>19:59</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>17</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>19</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>20:09</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>27</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>20:11</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>29</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>20:12</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>30</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>20:21</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>39</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>40</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>40</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>41</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>62</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>20:46</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>64</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>20:52</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>70</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>75</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>21:04</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>82</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>21:08</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>86</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>21:21</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>99</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -865,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -878,14 +1353,91 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:01:27</t>
+          <t>Última actualización: 19:42:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Ejecuciones: 0 filas únicas</t>
+          <t>Total filas: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Línea</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>41</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>19:42:45</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>21:08</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>86</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -900,7 +1452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -913,14 +1465,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:01:27</t>
+          <t>Última actualización: 19:42:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Ejecuciones: 2 filas únicas</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -996,6 +1548,56 @@
         <v>68</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>19:42:49</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>19:53</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>11</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>19:42:52</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>57</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>